<commit_message>
feat: update 'cadastrar_tomador' method with new XPaths and improved error handling
</commit_message>
<xml_diff>
--- a/notas_fiscais.xlsx
+++ b/notas_fiscais.xlsx
@@ -3270,16 +3270,20 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr"/>
-      <c r="K52" t="inlineStr"/>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Erro ao selecionar atividade</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:54</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr">
         <is>
           <t>04/02/2026</t>
@@ -3323,14 +3327,22 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr"/>
-      <c r="K53" t="inlineStr"/>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:57</t>
+        </is>
+      </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Erro ao cadastrar tomador</t>
+          <t>Erro ao selecionar atividade</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -3372,11 +3384,19 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr"/>
-      <c r="K54" t="inlineStr"/>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:57</t>
+        </is>
+      </c>
       <c r="L54" t="inlineStr">
         <is>
           <t>Erro ao cadastrar tomador</t>
@@ -3425,14 +3445,22 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J55" t="inlineStr"/>
-      <c r="K55" t="inlineStr"/>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:57</t>
+        </is>
+      </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Erro ao cadastrar tomador</t>
+          <t>Erro ao selecionar atividade</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -3478,16 +3506,20 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J56" t="inlineStr"/>
-      <c r="K56" t="inlineStr"/>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:57</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -3527,14 +3559,22 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J57" t="inlineStr"/>
-      <c r="K57" t="inlineStr"/>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>12/02/2026 17:57</t>
+        </is>
+      </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Erro ao cadastrar tomador</t>
+          <t>Erro ao selecionar atividade</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -3580,16 +3620,20 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J58" t="inlineStr"/>
-      <c r="K58" t="inlineStr"/>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:42</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -3633,16 +3677,20 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr"/>
-      <c r="K59" t="inlineStr"/>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:44</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr">
         <is>
           <t>05/02/2026</t>
@@ -3690,16 +3738,20 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr"/>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:46</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -3743,16 +3795,20 @@
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr"/>
-      <c r="K61" t="inlineStr"/>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:48</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr">
         <is>
           <t>07/02/2026</t>
@@ -4122,16 +4178,20 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J68" t="inlineStr"/>
-      <c r="K68" t="inlineStr"/>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>Erro ao selecionar atividade</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:50</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -4171,16 +4231,20 @@
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J69" t="inlineStr"/>
-      <c r="K69" t="inlineStr"/>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>Erro ao selecionar atividade</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:51</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -4228,16 +4292,20 @@
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J70" t="inlineStr"/>
-      <c r="K70" t="inlineStr"/>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:53</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr">
         <is>
           <t>05/02/2026</t>
@@ -4342,16 +4410,20 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J72" t="inlineStr"/>
-      <c r="K72" t="inlineStr"/>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>Erro ao selecionar atividade</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:55</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr">
         <is>
           <t>02/02/2026</t>
@@ -4391,16 +4463,20 @@
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr"/>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>Erro ao cadastrar tomador</t>
-        </is>
-      </c>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:57</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr">
         <is>
           <t>02/02/2026</t>
@@ -4438,9 +4514,21 @@
       <c r="H74" t="n">
         <v>110</v>
       </c>
-      <c r="I74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
-      <c r="K74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>12/02/2026 19:59</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr">
         <is>
@@ -4479,9 +4567,21 @@
       <c r="H75" t="n">
         <v>110</v>
       </c>
-      <c r="I75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
-      <c r="K75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:01</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr">
         <is>
@@ -4524,9 +4624,21 @@
       <c r="H76" t="n">
         <v>110</v>
       </c>
-      <c r="I76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:03</t>
+        </is>
+      </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr">
         <is>
@@ -4565,9 +4677,21 @@
       <c r="H77" t="n">
         <v>110</v>
       </c>
-      <c r="I77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
-      <c r="K77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:05</t>
+        </is>
+      </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr">
         <is>
@@ -4610,9 +4734,21 @@
       <c r="H78" t="n">
         <v>110</v>
       </c>
-      <c r="I78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
-      <c r="K78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:06</t>
+        </is>
+      </c>
       <c r="L78" t="inlineStr"/>
       <c r="M78" t="inlineStr">
         <is>
@@ -4655,9 +4791,21 @@
       <c r="H79" t="n">
         <v>110</v>
       </c>
-      <c r="I79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
-      <c r="K79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:08</t>
+        </is>
+      </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr">
         <is>
@@ -4696,9 +4844,21 @@
       <c r="H80" t="n">
         <v>110</v>
       </c>
-      <c r="I80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
-      <c r="K80" t="inlineStr"/>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:38</t>
+        </is>
+      </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr">
         <is>
@@ -4745,9 +4905,21 @@
       <c r="H81" t="n">
         <v>110</v>
       </c>
-      <c r="I81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
-      <c r="K81" t="inlineStr"/>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:40</t>
+        </is>
+      </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr">
         <is>
@@ -4786,9 +4958,21 @@
       <c r="H82" t="n">
         <v>110</v>
       </c>
-      <c r="I82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
-      <c r="K82" t="inlineStr"/>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:11</t>
+        </is>
+      </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr">
         <is>
@@ -4831,9 +5015,21 @@
       <c r="H83" t="n">
         <v>110</v>
       </c>
-      <c r="I83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
-      <c r="K83" t="inlineStr"/>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:13</t>
+        </is>
+      </c>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr">
         <is>
@@ -4876,9 +5072,21 @@
       <c r="H84" t="n">
         <v>110</v>
       </c>
-      <c r="I84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
-      <c r="K84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:14</t>
+        </is>
+      </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr">
         <is>
@@ -4917,9 +5125,21 @@
       <c r="H85" t="n">
         <v>110</v>
       </c>
-      <c r="I85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:16</t>
+        </is>
+      </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr">
         <is>
@@ -4958,9 +5178,21 @@
       <c r="H86" t="n">
         <v>110</v>
       </c>
-      <c r="I86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
-      <c r="K86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:18</t>
+        </is>
+      </c>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
@@ -4999,9 +5231,21 @@
       <c r="H87" t="n">
         <v>110</v>
       </c>
-      <c r="I87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
-      <c r="K87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:20</t>
+        </is>
+      </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
@@ -5044,9 +5288,21 @@
       <c r="H88" t="n">
         <v>110</v>
       </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
-      <c r="K88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:22</t>
+        </is>
+      </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
@@ -5089,9 +5345,21 @@
       <c r="H89" t="n">
         <v>110</v>
       </c>
-      <c r="I89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
-      <c r="K89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:24</t>
+        </is>
+      </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr">
         <is>
@@ -5130,9 +5398,21 @@
       <c r="H90" t="n">
         <v>110</v>
       </c>
-      <c r="I90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
-      <c r="K90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:26</t>
+        </is>
+      </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
@@ -5175,9 +5455,21 @@
       <c r="H91" t="n">
         <v>110</v>
       </c>
-      <c r="I91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
-      <c r="K91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:28</t>
+        </is>
+      </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
@@ -5216,9 +5508,21 @@
       <c r="H92" t="n">
         <v>110</v>
       </c>
-      <c r="I92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
-      <c r="K92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:30</t>
+        </is>
+      </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr">
         <is>
@@ -5261,9 +5565,21 @@
       <c r="H93" t="n">
         <v>110</v>
       </c>
-      <c r="I93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
-      <c r="K93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:42</t>
+        </is>
+      </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
@@ -5302,9 +5618,21 @@
       <c r="H94" t="n">
         <v>110</v>
       </c>
-      <c r="I94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
-      <c r="K94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:44</t>
+        </is>
+      </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
@@ -5347,9 +5675,21 @@
       <c r="H95" t="n">
         <v>110</v>
       </c>
-      <c r="I95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
-      <c r="K95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:46</t>
+        </is>
+      </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr">
         <is>
@@ -5388,9 +5728,21 @@
       <c r="H96" t="n">
         <v>110</v>
       </c>
-      <c r="I96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
-      <c r="K96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:48</t>
+        </is>
+      </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr">
         <is>
@@ -5433,9 +5785,21 @@
       <c r="H97" t="n">
         <v>110</v>
       </c>
-      <c r="I97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
-      <c r="K97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:50</t>
+        </is>
+      </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr">
         <is>
@@ -5474,9 +5838,21 @@
       <c r="H98" t="n">
         <v>110</v>
       </c>
-      <c r="I98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
-      <c r="K98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:52</t>
+        </is>
+      </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr">
         <is>
@@ -5515,9 +5891,21 @@
       <c r="H99" t="n">
         <v>110</v>
       </c>
-      <c r="I99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
-      <c r="K99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:53</t>
+        </is>
+      </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr">
         <is>
@@ -5560,9 +5948,21 @@
       <c r="H100" t="n">
         <v>110</v>
       </c>
-      <c r="I100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
-      <c r="K100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>12/02/2026 20:55</t>
+        </is>
+      </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr">
         <is>
@@ -5605,9 +6005,21 @@
       <c r="H101" t="n">
         <v>110</v>
       </c>
-      <c r="I101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
-      <c r="K101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>24/02/2026 19:39</t>
+        </is>
+      </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr">
         <is>
@@ -5650,9 +6062,21 @@
       <c r="H102" t="n">
         <v>110</v>
       </c>
-      <c r="I102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
-      <c r="K102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>24/02/2026 19:41</t>
+        </is>
+      </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr">
         <is>
@@ -5691,9 +6115,21 @@
       <c r="H103" t="n">
         <v>110</v>
       </c>
-      <c r="I103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
-      <c r="K103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>24/02/2026 19:41</t>
+        </is>
+      </c>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr">
         <is>
@@ -5732,9 +6168,21 @@
       <c r="H104" t="n">
         <v>110</v>
       </c>
-      <c r="I104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
-      <c r="K104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>24/02/2026 19:41</t>
+        </is>
+      </c>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr">
         <is>
@@ -5773,9 +6221,21 @@
       <c r="H105" t="n">
         <v>110</v>
       </c>
-      <c r="I105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
-      <c r="K105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:30</t>
+        </is>
+      </c>
       <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
@@ -5814,9 +6274,21 @@
       <c r="H106" t="n">
         <v>110</v>
       </c>
-      <c r="I106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
-      <c r="K106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:33</t>
+        </is>
+      </c>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr">
         <is>
@@ -5855,9 +6327,21 @@
       <c r="H107" t="n">
         <v>110</v>
       </c>
-      <c r="I107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
-      <c r="K107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:34</t>
+        </is>
+      </c>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr">
         <is>
@@ -5900,9 +6384,21 @@
       <c r="H108" t="n">
         <v>110</v>
       </c>
-      <c r="I108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
-      <c r="K108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:36</t>
+        </is>
+      </c>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr">
         <is>
@@ -5945,9 +6441,21 @@
       <c r="H109" t="n">
         <v>110</v>
       </c>
-      <c r="I109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
-      <c r="K109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:38</t>
+        </is>
+      </c>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr">
         <is>
@@ -5990,9 +6498,21 @@
       <c r="H110" t="n">
         <v>110</v>
       </c>
-      <c r="I110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
-      <c r="K110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:40</t>
+        </is>
+      </c>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr">
         <is>
@@ -6031,9 +6551,21 @@
       <c r="H111" t="n">
         <v>110</v>
       </c>
-      <c r="I111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
-      <c r="K111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:42</t>
+        </is>
+      </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr">
         <is>
@@ -6072,9 +6604,21 @@
       <c r="H112" t="n">
         <v>110</v>
       </c>
-      <c r="I112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
-      <c r="K112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:43</t>
+        </is>
+      </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr">
         <is>
@@ -6113,9 +6657,21 @@
       <c r="H113" t="n">
         <v>110</v>
       </c>
-      <c r="I113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
-      <c r="K113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:48</t>
+        </is>
+      </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr">
         <is>
@@ -6154,9 +6710,21 @@
       <c r="H114" t="n">
         <v>110</v>
       </c>
-      <c r="I114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
-      <c r="K114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:50</t>
+        </is>
+      </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr">
         <is>
@@ -6195,9 +6763,21 @@
       <c r="H115" t="n">
         <v>110</v>
       </c>
-      <c r="I115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
-      <c r="K115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:52</t>
+        </is>
+      </c>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr">
         <is>
@@ -6236,9 +6816,21 @@
       <c r="H116" t="n">
         <v>110</v>
       </c>
-      <c r="I116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
-      <c r="K116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:55</t>
+        </is>
+      </c>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr">
         <is>
@@ -6281,9 +6873,21 @@
       <c r="H117" t="n">
         <v>110</v>
       </c>
-      <c r="I117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
-      <c r="K117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:57</t>
+        </is>
+      </c>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr">
         <is>
@@ -6326,9 +6930,21 @@
       <c r="H118" t="n">
         <v>110</v>
       </c>
-      <c r="I118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
-      <c r="K118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>25/02/2026 18:58</t>
+        </is>
+      </c>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr">
         <is>
@@ -6371,9 +6987,21 @@
       <c r="H119" t="n">
         <v>110</v>
       </c>
-      <c r="I119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
-      <c r="K119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:07</t>
+        </is>
+      </c>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr">
         <is>
@@ -6412,9 +7040,21 @@
       <c r="H120" t="n">
         <v>110</v>
       </c>
-      <c r="I120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
-      <c r="K120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:09</t>
+        </is>
+      </c>
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr">
         <is>
@@ -6453,9 +7093,21 @@
       <c r="H121" t="n">
         <v>110</v>
       </c>
-      <c r="I121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
-      <c r="K121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:11</t>
+        </is>
+      </c>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr">
         <is>
@@ -6494,9 +7146,21 @@
       <c r="H122" t="n">
         <v>110</v>
       </c>
-      <c r="I122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
-      <c r="K122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:19</t>
+        </is>
+      </c>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr">
         <is>
@@ -6539,9 +7203,21 @@
       <c r="H123" t="n">
         <v>110</v>
       </c>
-      <c r="I123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-      <c r="K123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:19</t>
+        </is>
+      </c>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr">
         <is>
@@ -6580,9 +7256,21 @@
       <c r="H124" t="n">
         <v>110</v>
       </c>
-      <c r="I124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-      <c r="K124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:26</t>
+        </is>
+      </c>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr">
         <is>
@@ -6625,9 +7313,21 @@
       <c r="H125" t="n">
         <v>110</v>
       </c>
-      <c r="I125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-      <c r="K125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:29</t>
+        </is>
+      </c>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr">
         <is>
@@ -6670,9 +7370,21 @@
       <c r="H126" t="n">
         <v>110</v>
       </c>
-      <c r="I126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-      <c r="K126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:31</t>
+        </is>
+      </c>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr">
         <is>
@@ -6715,9 +7427,21 @@
       <c r="H127" t="n">
         <v>110</v>
       </c>
-      <c r="I127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-      <c r="K127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:33</t>
+        </is>
+      </c>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr">
         <is>
@@ -6764,9 +7488,21 @@
       <c r="H128" t="n">
         <v>110</v>
       </c>
-      <c r="I128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-      <c r="K128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:41</t>
+        </is>
+      </c>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr">
         <is>
@@ -6805,9 +7541,21 @@
       <c r="H129" t="n">
         <v>110</v>
       </c>
-      <c r="I129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-      <c r="K129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:43</t>
+        </is>
+      </c>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr">
         <is>
@@ -6850,9 +7598,21 @@
       <c r="H130" t="n">
         <v>110</v>
       </c>
-      <c r="I130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-      <c r="K130" t="inlineStr"/>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:46</t>
+        </is>
+      </c>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr">
         <is>
@@ -6891,9 +7651,21 @@
       <c r="H131" t="n">
         <v>110</v>
       </c>
-      <c r="I131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-      <c r="K131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:48</t>
+        </is>
+      </c>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr">
         <is>
@@ -6936,9 +7708,21 @@
       <c r="H132" t="n">
         <v>110</v>
       </c>
-      <c r="I132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-      <c r="K132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:50</t>
+        </is>
+      </c>
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr">
         <is>
@@ -6981,9 +7765,21 @@
       <c r="H133" t="n">
         <v>110</v>
       </c>
-      <c r="I133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-      <c r="K133" t="inlineStr"/>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:52</t>
+        </is>
+      </c>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr">
         <is>
@@ -7022,9 +7818,21 @@
       <c r="H134" t="n">
         <v>110</v>
       </c>
-      <c r="I134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-      <c r="K134" t="inlineStr"/>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:55</t>
+        </is>
+      </c>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr">
         <is>
@@ -7067,9 +7875,21 @@
       <c r="H135" t="n">
         <v>110</v>
       </c>
-      <c r="I135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
-      <c r="K135" t="inlineStr"/>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:57</t>
+        </is>
+      </c>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr">
         <is>
@@ -7108,9 +7928,21 @@
       <c r="H136" t="n">
         <v>110</v>
       </c>
-      <c r="I136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-      <c r="K136" t="inlineStr"/>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>25/02/2026 19:59</t>
+        </is>
+      </c>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr">
         <is>
@@ -7149,9 +7981,21 @@
       <c r="H137" t="n">
         <v>110</v>
       </c>
-      <c r="I137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-      <c r="K137" t="inlineStr"/>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:02</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr">
         <is>
@@ -7190,9 +8034,21 @@
       <c r="H138" t="n">
         <v>110</v>
       </c>
-      <c r="I138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
-      <c r="K138" t="inlineStr"/>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:04</t>
+        </is>
+      </c>
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr">
         <is>
@@ -7235,9 +8091,21 @@
       <c r="H139" t="n">
         <v>110</v>
       </c>
-      <c r="I139" t="inlineStr"/>
-      <c r="J139" t="inlineStr"/>
-      <c r="K139" t="inlineStr"/>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:09</t>
+        </is>
+      </c>
       <c r="L139" t="inlineStr"/>
       <c r="M139" t="inlineStr">
         <is>
@@ -7276,9 +8144,21 @@
       <c r="H140" t="n">
         <v>110</v>
       </c>
-      <c r="I140" t="inlineStr"/>
-      <c r="J140" t="inlineStr"/>
-      <c r="K140" t="inlineStr"/>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:11</t>
+        </is>
+      </c>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr">
         <is>
@@ -7321,9 +8201,21 @@
       <c r="H141" t="n">
         <v>110</v>
       </c>
-      <c r="I141" t="inlineStr"/>
-      <c r="J141" t="inlineStr"/>
-      <c r="K141" t="inlineStr"/>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:15</t>
+        </is>
+      </c>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr">
         <is>
@@ -7362,9 +8254,21 @@
       <c r="H142" t="n">
         <v>110</v>
       </c>
-      <c r="I142" t="inlineStr"/>
-      <c r="J142" t="inlineStr"/>
-      <c r="K142" t="inlineStr"/>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:18</t>
+        </is>
+      </c>
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr">
         <is>
@@ -7407,9 +8311,21 @@
       <c r="H143" t="n">
         <v>110</v>
       </c>
-      <c r="I143" t="inlineStr"/>
-      <c r="J143" t="inlineStr"/>
-      <c r="K143" t="inlineStr"/>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:20</t>
+        </is>
+      </c>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr">
         <is>
@@ -7448,9 +8364,21 @@
       <c r="H144" t="n">
         <v>110</v>
       </c>
-      <c r="I144" t="inlineStr"/>
-      <c r="J144" t="inlineStr"/>
-      <c r="K144" t="inlineStr"/>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:22</t>
+        </is>
+      </c>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr">
         <is>
@@ -7497,9 +8425,21 @@
       <c r="H145" t="n">
         <v>110</v>
       </c>
-      <c r="I145" t="inlineStr"/>
-      <c r="J145" t="inlineStr"/>
-      <c r="K145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:24</t>
+        </is>
+      </c>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr">
         <is>
@@ -7538,9 +8478,21 @@
       <c r="H146" t="n">
         <v>110</v>
       </c>
-      <c r="I146" t="inlineStr"/>
-      <c r="J146" t="inlineStr"/>
-      <c r="K146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:25</t>
+        </is>
+      </c>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr">
         <is>
@@ -7583,9 +8535,21 @@
       <c r="H147" t="n">
         <v>110</v>
       </c>
-      <c r="I147" t="inlineStr"/>
-      <c r="J147" t="inlineStr"/>
-      <c r="K147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:27</t>
+        </is>
+      </c>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr">
         <is>
@@ -7624,9 +8588,21 @@
       <c r="H148" t="n">
         <v>110</v>
       </c>
-      <c r="I148" t="inlineStr"/>
-      <c r="J148" t="inlineStr"/>
-      <c r="K148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:29</t>
+        </is>
+      </c>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr">
         <is>
@@ -7665,9 +8641,21 @@
       <c r="H149" t="n">
         <v>110</v>
       </c>
-      <c r="I149" t="inlineStr"/>
-      <c r="J149" t="inlineStr"/>
-      <c r="K149" t="inlineStr"/>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:36</t>
+        </is>
+      </c>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr">
         <is>
@@ -7710,9 +8698,21 @@
       <c r="H150" t="n">
         <v>110</v>
       </c>
-      <c r="I150" t="inlineStr"/>
-      <c r="J150" t="inlineStr"/>
-      <c r="K150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:38</t>
+        </is>
+      </c>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr">
         <is>
@@ -7751,9 +8751,21 @@
       <c r="H151" t="n">
         <v>110</v>
       </c>
-      <c r="I151" t="inlineStr"/>
-      <c r="J151" t="inlineStr"/>
-      <c r="K151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:40</t>
+        </is>
+      </c>
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr">
         <is>
@@ -7796,9 +8808,21 @@
       <c r="H152" t="n">
         <v>110</v>
       </c>
-      <c r="I152" t="inlineStr"/>
-      <c r="J152" t="inlineStr"/>
-      <c r="K152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:42</t>
+        </is>
+      </c>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr">
         <is>
@@ -7837,9 +8861,21 @@
       <c r="H153" t="n">
         <v>110</v>
       </c>
-      <c r="I153" t="inlineStr"/>
-      <c r="J153" t="inlineStr"/>
-      <c r="K153" t="inlineStr"/>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:44</t>
+        </is>
+      </c>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr">
         <is>
@@ -7878,9 +8914,21 @@
       <c r="H154" t="n">
         <v>110</v>
       </c>
-      <c r="I154" t="inlineStr"/>
-      <c r="J154" t="inlineStr"/>
-      <c r="K154" t="inlineStr"/>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:46</t>
+        </is>
+      </c>
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr">
         <is>
@@ -7919,9 +8967,21 @@
       <c r="H155" t="n">
         <v>110</v>
       </c>
-      <c r="I155" t="inlineStr"/>
-      <c r="J155" t="inlineStr"/>
-      <c r="K155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:48</t>
+        </is>
+      </c>
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr">
         <is>
@@ -7960,9 +9020,21 @@
       <c r="H156" t="n">
         <v>110</v>
       </c>
-      <c r="I156" t="inlineStr"/>
-      <c r="J156" t="inlineStr"/>
-      <c r="K156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:50</t>
+        </is>
+      </c>
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr">
         <is>
@@ -8001,9 +9073,21 @@
       <c r="H157" t="n">
         <v>110</v>
       </c>
-      <c r="I157" t="inlineStr"/>
-      <c r="J157" t="inlineStr"/>
-      <c r="K157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:52</t>
+        </is>
+      </c>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr">
         <is>
@@ -8042,9 +9126,21 @@
       <c r="H158" t="n">
         <v>110</v>
       </c>
-      <c r="I158" t="inlineStr"/>
-      <c r="J158" t="inlineStr"/>
-      <c r="K158" t="inlineStr"/>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:54</t>
+        </is>
+      </c>
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr">
         <is>
@@ -8083,9 +9179,21 @@
       <c r="H159" t="n">
         <v>110</v>
       </c>
-      <c r="I159" t="inlineStr"/>
-      <c r="J159" t="inlineStr"/>
-      <c r="K159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:56</t>
+        </is>
+      </c>
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr">
         <is>
@@ -8124,9 +9232,21 @@
       <c r="H160" t="n">
         <v>110</v>
       </c>
-      <c r="I160" t="inlineStr"/>
-      <c r="J160" t="inlineStr"/>
-      <c r="K160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Emitida</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>25/02/2026 20:58</t>
+        </is>
+      </c>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr">
         <is>
@@ -8169,10 +9289,18 @@
       <c r="H161" t="n">
         <v>110</v>
       </c>
-      <c r="I161" t="inlineStr"/>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J161" t="inlineStr"/>
       <c r="K161" t="inlineStr"/>
-      <c r="L161" t="inlineStr"/>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M161" t="inlineStr">
         <is>
           <t>06/02/2026</t>
@@ -8214,10 +9342,18 @@
       <c r="H162" t="n">
         <v>110</v>
       </c>
-      <c r="I162" t="inlineStr"/>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J162" t="inlineStr"/>
       <c r="K162" t="inlineStr"/>
-      <c r="L162" t="inlineStr"/>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M162" t="inlineStr">
         <is>
           <t>06/02/2026</t>
@@ -8263,10 +9399,18 @@
       <c r="H163" t="n">
         <v>110</v>
       </c>
-      <c r="I163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J163" t="inlineStr"/>
       <c r="K163" t="inlineStr"/>
-      <c r="L163" t="inlineStr"/>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M163" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -8308,10 +9452,18 @@
       <c r="H164" t="n">
         <v>110</v>
       </c>
-      <c r="I164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J164" t="inlineStr"/>
       <c r="K164" t="inlineStr"/>
-      <c r="L164" t="inlineStr"/>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M164" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -8353,10 +9505,18 @@
       <c r="H165" t="n">
         <v>110</v>
       </c>
-      <c r="I165" t="inlineStr"/>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J165" t="inlineStr"/>
       <c r="K165" t="inlineStr"/>
-      <c r="L165" t="inlineStr"/>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M165" t="inlineStr">
         <is>
           <t>04/02/2026</t>
@@ -8398,10 +9558,18 @@
       <c r="H166" t="n">
         <v>110</v>
       </c>
-      <c r="I166" t="inlineStr"/>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J166" t="inlineStr"/>
       <c r="K166" t="inlineStr"/>
-      <c r="L166" t="inlineStr"/>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M166" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -8439,10 +9607,18 @@
       <c r="H167" t="n">
         <v>110</v>
       </c>
-      <c r="I167" t="inlineStr"/>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J167" t="inlineStr"/>
       <c r="K167" t="inlineStr"/>
-      <c r="L167" t="inlineStr"/>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M167" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -8488,10 +9664,18 @@
       <c r="H168" t="n">
         <v>110</v>
       </c>
-      <c r="I168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J168" t="inlineStr"/>
       <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M168" t="inlineStr">
         <is>
           <t>09/02/2026</t>
@@ -8529,10 +9713,18 @@
       <c r="H169" t="n">
         <v>110</v>
       </c>
-      <c r="I169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J169" t="inlineStr"/>
       <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M169" t="inlineStr">
         <is>
           <t>02/02/2026</t>
@@ -8570,10 +9762,18 @@
       <c r="H170" t="n">
         <v>110</v>
       </c>
-      <c r="I170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J170" t="inlineStr"/>
       <c r="K170" t="inlineStr"/>
-      <c r="L170" t="inlineStr"/>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M170" t="inlineStr">
         <is>
           <t>27/02/2026</t>
@@ -8611,10 +9811,18 @@
       <c r="H171" t="n">
         <v>110</v>
       </c>
-      <c r="I171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J171" t="inlineStr"/>
       <c r="K171" t="inlineStr"/>
-      <c r="L171" t="inlineStr"/>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M171" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -8652,10 +9860,18 @@
       <c r="H172" t="n">
         <v>110</v>
       </c>
-      <c r="I172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J172" t="inlineStr"/>
       <c r="K172" t="inlineStr"/>
-      <c r="L172" t="inlineStr"/>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M172" t="inlineStr">
         <is>
           <t>28/02/2026</t>
@@ -8697,10 +9913,18 @@
       <c r="H173" t="n">
         <v>110</v>
       </c>
-      <c r="I173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr"/>
       <c r="K173" t="inlineStr"/>
-      <c r="L173" t="inlineStr"/>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M173" t="inlineStr">
         <is>
           <t>01/02/2026</t>
@@ -8746,10 +9970,18 @@
       <c r="H174" t="n">
         <v>110</v>
       </c>
-      <c r="I174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J174" t="inlineStr"/>
       <c r="K174" t="inlineStr"/>
-      <c r="L174" t="inlineStr"/>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M174" t="inlineStr">
         <is>
           <t>05/02/2026</t>
@@ -8791,10 +10023,18 @@
       <c r="H175" t="n">
         <v>110</v>
       </c>
-      <c r="I175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J175" t="inlineStr"/>
       <c r="K175" t="inlineStr"/>
-      <c r="L175" t="inlineStr"/>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M175" t="inlineStr">
         <is>
           <t>05/02/2026</t>
@@ -8828,10 +10068,18 @@
       <c r="H176" t="n">
         <v>110</v>
       </c>
-      <c r="I176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J176" t="inlineStr"/>
       <c r="K176" t="inlineStr"/>
-      <c r="L176" t="inlineStr"/>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M176" t="inlineStr">
         <is>
           <t>10/02/2026</t>
@@ -8869,10 +10117,18 @@
       <c r="H177" t="n">
         <v>110</v>
       </c>
-      <c r="I177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr"/>
       <c r="K177" t="inlineStr"/>
-      <c r="L177" t="inlineStr"/>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M177" t="inlineStr">
         <is>
           <t>02/02/2026</t>
@@ -8910,10 +10166,18 @@
       <c r="H178" t="n">
         <v>110</v>
       </c>
-      <c r="I178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>ERRO</t>
+        </is>
+      </c>
       <c r="J178" t="inlineStr"/>
       <c r="K178" t="inlineStr"/>
-      <c r="L178" t="inlineStr"/>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>Erro ao pesquisar CPF</t>
+        </is>
+      </c>
       <c r="M178" t="inlineStr">
         <is>
           <t>02/02/2026</t>

</xml_diff>